<commit_message>
Add 4 new terms: hit the roof, cold as ice, lie through one's teeth, backbone
</commit_message>
<xml_diff>
--- a/excel/EnglishTerms.xlsx
+++ b/excel/EnglishTerms.xlsx
@@ -7118,40 +7118,104 @@
       <c r="H260" s="8" t="n"/>
     </row>
     <row r="261">
-      <c r="A261" s="8" t="n"/>
-      <c r="B261" s="8" t="n"/>
-      <c r="C261" s="7" t="n"/>
-      <c r="D261" s="8" t="n"/>
+      <c r="A261" s="8" t="inlineStr">
+        <is>
+          <t>hit the roof</t>
+        </is>
+      </c>
+      <c r="B261" s="8" t="inlineStr">
+        <is>
+          <t>to suddenly become very angry</t>
+        </is>
+      </c>
+      <c r="C261" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D261" s="8" t="inlineStr">
+        <is>
+          <t>Dad hit the roof when he saw the dent in the car.</t>
+        </is>
+      </c>
       <c r="E261" s="8" t="n"/>
       <c r="F261" s="9" t="n"/>
       <c r="G261" s="7" t="n"/>
       <c r="H261" s="8" t="n"/>
     </row>
     <row r="262">
-      <c r="A262" s="8" t="n"/>
-      <c r="B262" s="8" t="n"/>
-      <c r="C262" s="7" t="n"/>
-      <c r="D262" s="8" t="n"/>
+      <c r="A262" s="8" t="inlineStr">
+        <is>
+          <t>cold as ice</t>
+        </is>
+      </c>
+      <c r="B262" s="8" t="inlineStr">
+        <is>
+          <t>extremely cold in temperature, or emotionally distant and unfriendly</t>
+        </is>
+      </c>
+      <c r="C262" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D262" s="8" t="inlineStr">
+        <is>
+          <t>Her hands were cold as ice after walking home in the snow.</t>
+        </is>
+      </c>
       <c r="E262" s="8" t="n"/>
       <c r="F262" s="9" t="n"/>
       <c r="G262" s="7" t="n"/>
       <c r="H262" s="8" t="n"/>
     </row>
     <row r="263">
-      <c r="A263" s="8" t="n"/>
-      <c r="B263" s="8" t="n"/>
-      <c r="C263" s="7" t="n"/>
-      <c r="D263" s="8" t="n"/>
+      <c r="A263" s="8" t="inlineStr">
+        <is>
+          <t>to lie through one’s teeth</t>
+        </is>
+      </c>
+      <c r="B263" s="8" t="inlineStr">
+        <is>
+          <t>to tell a blatant, shameless lie while knowing it is completely untrue</t>
+        </is>
+      </c>
+      <c r="C263" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D263" s="8" t="inlineStr">
+        <is>
+          <t>He was lying through his teeth when he said he had never met her before.</t>
+        </is>
+      </c>
       <c r="E263" s="8" t="n"/>
       <c r="F263" s="9" t="n"/>
       <c r="G263" s="7" t="n"/>
       <c r="H263" s="8" t="n"/>
     </row>
     <row r="264">
-      <c r="A264" s="8" t="n"/>
-      <c r="B264" s="8" t="n"/>
-      <c r="C264" s="7" t="n"/>
-      <c r="D264" s="8" t="n"/>
+      <c r="A264" s="8" t="inlineStr">
+        <is>
+          <t>backbone</t>
+        </is>
+      </c>
+      <c r="B264" s="8" t="inlineStr">
+        <is>
+          <t>the spine; figuratively, the strength of character or the main support of something</t>
+        </is>
+      </c>
+      <c r="C264" s="7" t="inlineStr">
+        <is>
+          <t>vocab</t>
+        </is>
+      </c>
+      <c r="D264" s="8" t="inlineStr">
+        <is>
+          <t>It takes real backbone to stand up to a bully at school.</t>
+        </is>
+      </c>
       <c r="E264" s="8" t="n"/>
       <c r="F264" s="9" t="n"/>
       <c r="G264" s="7" t="n"/>

</xml_diff>

<commit_message>
Add 6 idioms from wheel: sweating buckets, about to explode, fly off the handle, full of beans, white lie, hot air
</commit_message>
<xml_diff>
--- a/excel/EnglishTerms.xlsx
+++ b/excel/EnglishTerms.xlsx
@@ -7222,60 +7222,156 @@
       <c r="H264" s="8" t="n"/>
     </row>
     <row r="265">
-      <c r="A265" s="8" t="n"/>
-      <c r="B265" s="8" t="n"/>
-      <c r="C265" s="7" t="n"/>
-      <c r="D265" s="8" t="n"/>
+      <c r="A265" s="8" t="inlineStr">
+        <is>
+          <t>sweating buckets</t>
+        </is>
+      </c>
+      <c r="B265" s="8" t="inlineStr">
+        <is>
+          <t>sweating profusely, usually from heat, exertion, or nervousness</t>
+        </is>
+      </c>
+      <c r="C265" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D265" s="8" t="inlineStr">
+        <is>
+          <t>I was sweating buckets during the job interview.</t>
+        </is>
+      </c>
       <c r="E265" s="8" t="n"/>
       <c r="F265" s="9" t="n"/>
       <c r="G265" s="7" t="n"/>
       <c r="H265" s="8" t="n"/>
     </row>
     <row r="266">
-      <c r="A266" s="8" t="n"/>
-      <c r="B266" s="8" t="n"/>
-      <c r="C266" s="7" t="n"/>
-      <c r="D266" s="8" t="n"/>
+      <c r="A266" s="8" t="inlineStr">
+        <is>
+          <t>about to explode</t>
+        </is>
+      </c>
+      <c r="B266" s="8" t="inlineStr">
+        <is>
+          <t>on the verge of losing one’s temper or bursting with an intense emotion</t>
+        </is>
+      </c>
+      <c r="C266" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D266" s="8" t="inlineStr">
+        <is>
+          <t>After hours of traffic, I was about to explode.</t>
+        </is>
+      </c>
       <c r="E266" s="8" t="n"/>
       <c r="F266" s="9" t="n"/>
       <c r="G266" s="7" t="n"/>
       <c r="H266" s="8" t="n"/>
     </row>
     <row r="267">
-      <c r="A267" s="8" t="n"/>
-      <c r="B267" s="8" t="n"/>
-      <c r="C267" s="7" t="n"/>
-      <c r="D267" s="8" t="n"/>
+      <c r="A267" s="8" t="inlineStr">
+        <is>
+          <t>fly off the handle</t>
+        </is>
+      </c>
+      <c r="B267" s="8" t="inlineStr">
+        <is>
+          <t>to suddenly become very angry and lose self-control</t>
+        </is>
+      </c>
+      <c r="C267" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D267" s="8" t="inlineStr">
+        <is>
+          <t>He flew off the handle when he realized someone had dented his car.</t>
+        </is>
+      </c>
       <c r="E267" s="8" t="n"/>
       <c r="F267" s="9" t="n"/>
       <c r="G267" s="7" t="n"/>
       <c r="H267" s="8" t="n"/>
     </row>
     <row r="268">
-      <c r="A268" s="8" t="n"/>
-      <c r="B268" s="8" t="n"/>
-      <c r="C268" s="7" t="n"/>
-      <c r="D268" s="8" t="n"/>
+      <c r="A268" s="8" t="inlineStr">
+        <is>
+          <t>full of beans</t>
+        </is>
+      </c>
+      <c r="B268" s="8" t="inlineStr">
+        <is>
+          <t>full of energy, lively and enthusiastic</t>
+        </is>
+      </c>
+      <c r="C268" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D268" s="8" t="inlineStr">
+        <is>
+          <t>The kids were full of beans after eating all that candy.</t>
+        </is>
+      </c>
       <c r="E268" s="8" t="n"/>
       <c r="F268" s="9" t="n"/>
       <c r="G268" s="7" t="n"/>
       <c r="H268" s="8" t="n"/>
     </row>
     <row r="269">
-      <c r="A269" s="8" t="n"/>
-      <c r="B269" s="8" t="n"/>
-      <c r="C269" s="7" t="n"/>
-      <c r="D269" s="8" t="n"/>
+      <c r="A269" s="8" t="inlineStr">
+        <is>
+          <t>white lie</t>
+        </is>
+      </c>
+      <c r="B269" s="8" t="inlineStr">
+        <is>
+          <t>a small, harmless lie told to avoid hurting someone’s feelings or to be polite</t>
+        </is>
+      </c>
+      <c r="C269" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D269" s="8" t="inlineStr">
+        <is>
+          <t>She told a white lie and said she loved the gift.</t>
+        </is>
+      </c>
       <c r="E269" s="8" t="n"/>
       <c r="F269" s="9" t="n"/>
       <c r="G269" s="7" t="n"/>
       <c r="H269" s="8" t="n"/>
     </row>
     <row r="270">
-      <c r="A270" s="8" t="n"/>
-      <c r="B270" s="8" t="n"/>
-      <c r="C270" s="7" t="n"/>
-      <c r="D270" s="8" t="n"/>
+      <c r="A270" s="8" t="inlineStr">
+        <is>
+          <t>hot air</t>
+        </is>
+      </c>
+      <c r="B270" s="8" t="inlineStr">
+        <is>
+          <t>empty, boastful or meaningless talk that has no substance behind it</t>
+        </is>
+      </c>
+      <c r="C270" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D270" s="8" t="inlineStr">
+        <is>
+          <t>His promises are just hot air — he never actually does anything.</t>
+        </is>
+      </c>
       <c r="E270" s="8" t="n"/>
       <c r="F270" s="9" t="n"/>
       <c r="G270" s="7" t="n"/>

</xml_diff>

<commit_message>
Add 38 new terms: 4 adjectives + 34 common idioms from ProWritingAid
- Adjectives (vocab): Chilly, Harsh, Blunt, Dull
- Common idioms: a bed of roses, a blast from the past, a bolt from the blue,
  a drop in the bucket, a fish out of water, a no-brainer, a shot in the dark,
  a stone's throw away, a wolf in sheep's clothing, above board, actions speak
  louder than words, all ears, apple of my eye, at the drop of a hat, at the
  eleventh hour, back to square one, bend over backwards, better late than
  never, better safe than sorry, bite the dust, blow your mind, break a leg,
  bring home the bacon, burn the candle at both ends, bury the hatchet, by the
  skin of your teeth, call it a day, can of worms, catch-22, caught red-handed,
  chew the fat, clear the air, close call, cold turkey

Total terms: 269 -> 307
</commit_message>
<xml_diff>
--- a/excel/EnglishTerms.xlsx
+++ b/excel/EnglishTerms.xlsx
@@ -7378,380 +7378,988 @@
       <c r="H270" s="8" t="n"/>
     </row>
     <row r="271">
-      <c r="A271" s="8" t="n"/>
-      <c r="B271" s="8" t="n"/>
-      <c r="C271" s="7" t="n"/>
-      <c r="D271" s="8" t="n"/>
+      <c r="A271" s="8" t="inlineStr">
+        <is>
+          <t>Chilly</t>
+        </is>
+      </c>
+      <c r="B271" s="8" t="inlineStr">
+        <is>
+          <t>Unpleasantly cold; uncomfortably cool</t>
+        </is>
+      </c>
+      <c r="C271" s="7" t="inlineStr">
+        <is>
+          <t>vocab</t>
+        </is>
+      </c>
+      <c r="D271" s="8" t="inlineStr">
+        <is>
+          <t>The weather was chilly this morning, so I wore a sweater.</t>
+        </is>
+      </c>
       <c r="E271" s="8" t="n"/>
       <c r="F271" s="9" t="n"/>
       <c r="G271" s="7" t="n"/>
       <c r="H271" s="8" t="n"/>
     </row>
     <row r="272">
-      <c r="A272" s="8" t="n"/>
-      <c r="B272" s="8" t="n"/>
-      <c r="C272" s="7" t="n"/>
-      <c r="D272" s="8" t="n"/>
+      <c r="A272" s="8" t="inlineStr">
+        <is>
+          <t>Harsh</t>
+        </is>
+      </c>
+      <c r="B272" s="8" t="inlineStr">
+        <is>
+          <t>Unpleasantly rough, severe, or cruel</t>
+        </is>
+      </c>
+      <c r="C272" s="7" t="inlineStr">
+        <is>
+          <t>vocab</t>
+        </is>
+      </c>
+      <c r="D272" s="8" t="inlineStr">
+        <is>
+          <t>The teacher's harsh words made the student cry.</t>
+        </is>
+      </c>
       <c r="E272" s="8" t="n"/>
       <c r="F272" s="9" t="n"/>
       <c r="G272" s="7" t="n"/>
       <c r="H272" s="8" t="n"/>
     </row>
     <row r="273">
-      <c r="A273" s="8" t="n"/>
-      <c r="B273" s="8" t="n"/>
-      <c r="C273" s="7" t="n"/>
-      <c r="D273" s="8" t="n"/>
+      <c r="A273" s="8" t="inlineStr">
+        <is>
+          <t>Blunt</t>
+        </is>
+      </c>
+      <c r="B273" s="8" t="inlineStr">
+        <is>
+          <t>Direct and straightforward, sometimes to the point of rudeness</t>
+        </is>
+      </c>
+      <c r="C273" s="7" t="inlineStr">
+        <is>
+          <t>vocab</t>
+        </is>
+      </c>
+      <c r="D273" s="8" t="inlineStr">
+        <is>
+          <t>She was very blunt with her feedback about his work.</t>
+        </is>
+      </c>
       <c r="E273" s="8" t="n"/>
       <c r="F273" s="9" t="n"/>
       <c r="G273" s="7" t="n"/>
       <c r="H273" s="8" t="n"/>
     </row>
     <row r="274">
-      <c r="A274" s="8" t="n"/>
-      <c r="B274" s="8" t="n"/>
-      <c r="C274" s="7" t="n"/>
-      <c r="D274" s="8" t="n"/>
+      <c r="A274" s="8" t="inlineStr">
+        <is>
+          <t>Dull</t>
+        </is>
+      </c>
+      <c r="B274" s="8" t="inlineStr">
+        <is>
+          <t>Lacking excitement, brightness, or sharpness; boring</t>
+        </is>
+      </c>
+      <c r="C274" s="7" t="inlineStr">
+        <is>
+          <t>vocab</t>
+        </is>
+      </c>
+      <c r="D274" s="8" t="inlineStr">
+        <is>
+          <t>The lecture was so dull that I almost fell asleep.</t>
+        </is>
+      </c>
       <c r="E274" s="8" t="n"/>
       <c r="F274" s="9" t="n"/>
       <c r="G274" s="7" t="n"/>
       <c r="H274" s="8" t="n"/>
     </row>
     <row r="275">
-      <c r="A275" s="8" t="n"/>
-      <c r="B275" s="8" t="n"/>
-      <c r="C275" s="7" t="n"/>
-      <c r="D275" s="8" t="n"/>
+      <c r="A275" s="8" t="inlineStr">
+        <is>
+          <t>a bed of roses</t>
+        </is>
+      </c>
+      <c r="B275" s="8" t="inlineStr">
+        <is>
+          <t>An easy, comfortable situation with no problems</t>
+        </is>
+      </c>
+      <c r="C275" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D275" s="8" t="inlineStr">
+        <is>
+          <t>Being a CEO is not a bed of roses; it comes with many challenges.</t>
+        </is>
+      </c>
       <c r="E275" s="8" t="n"/>
       <c r="F275" s="9" t="n"/>
       <c r="G275" s="7" t="n"/>
       <c r="H275" s="8" t="n"/>
     </row>
     <row r="276">
-      <c r="A276" s="8" t="n"/>
-      <c r="B276" s="8" t="n"/>
-      <c r="C276" s="7" t="n"/>
-      <c r="D276" s="8" t="n"/>
+      <c r="A276" s="8" t="inlineStr">
+        <is>
+          <t>a blast from the past</t>
+        </is>
+      </c>
+      <c r="B276" s="8" t="inlineStr">
+        <is>
+          <t>Something or someone that reminds you of the past</t>
+        </is>
+      </c>
+      <c r="C276" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D276" s="8" t="inlineStr">
+        <is>
+          <t>Seeing my old school friend was a real blast from the past.</t>
+        </is>
+      </c>
       <c r="E276" s="8" t="n"/>
       <c r="F276" s="9" t="n"/>
       <c r="G276" s="7" t="n"/>
       <c r="H276" s="8" t="n"/>
     </row>
     <row r="277">
-      <c r="A277" s="8" t="n"/>
-      <c r="B277" s="8" t="n"/>
-      <c r="C277" s="7" t="n"/>
-      <c r="D277" s="8" t="n"/>
+      <c r="A277" s="8" t="inlineStr">
+        <is>
+          <t>a bolt from the blue</t>
+        </is>
+      </c>
+      <c r="B277" s="8" t="inlineStr">
+        <is>
+          <t>A sudden, unexpected event or news</t>
+        </is>
+      </c>
+      <c r="C277" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D277" s="8" t="inlineStr">
+        <is>
+          <t>Her resignation came as a bolt from the blue to everyone in the office.</t>
+        </is>
+      </c>
       <c r="E277" s="8" t="n"/>
       <c r="F277" s="9" t="n"/>
       <c r="G277" s="7" t="n"/>
       <c r="H277" s="8" t="n"/>
     </row>
     <row r="278">
-      <c r="A278" s="8" t="n"/>
-      <c r="B278" s="8" t="n"/>
-      <c r="C278" s="7" t="n"/>
-      <c r="D278" s="8" t="n"/>
+      <c r="A278" s="8" t="inlineStr">
+        <is>
+          <t>a drop in the bucket</t>
+        </is>
+      </c>
+      <c r="B278" s="8" t="inlineStr">
+        <is>
+          <t>A very small amount compared to what is needed</t>
+        </is>
+      </c>
+      <c r="C278" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D278" s="8" t="inlineStr">
+        <is>
+          <t>My donation is just a drop in the bucket, but every bit helps.</t>
+        </is>
+      </c>
       <c r="E278" s="8" t="n"/>
       <c r="F278" s="9" t="n"/>
       <c r="G278" s="7" t="n"/>
       <c r="H278" s="8" t="n"/>
     </row>
     <row r="279">
-      <c r="A279" s="8" t="n"/>
-      <c r="B279" s="8" t="n"/>
-      <c r="C279" s="7" t="n"/>
-      <c r="D279" s="8" t="n"/>
+      <c r="A279" s="8" t="inlineStr">
+        <is>
+          <t>a fish out of water</t>
+        </is>
+      </c>
+      <c r="B279" s="8" t="inlineStr">
+        <is>
+          <t>Someone who feels uncomfortable in an unfamiliar situation</t>
+        </is>
+      </c>
+      <c r="C279" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D279" s="8" t="inlineStr">
+        <is>
+          <t>At the fancy party, I felt like a fish out of water.</t>
+        </is>
+      </c>
       <c r="E279" s="8" t="n"/>
       <c r="F279" s="9" t="n"/>
       <c r="G279" s="7" t="n"/>
       <c r="H279" s="8" t="n"/>
     </row>
     <row r="280">
-      <c r="A280" s="8" t="n"/>
-      <c r="B280" s="8" t="n"/>
-      <c r="C280" s="7" t="n"/>
-      <c r="D280" s="8" t="n"/>
+      <c r="A280" s="8" t="inlineStr">
+        <is>
+          <t>a no-brainer</t>
+        </is>
+      </c>
+      <c r="B280" s="8" t="inlineStr">
+        <is>
+          <t>An easy decision; something obvious</t>
+        </is>
+      </c>
+      <c r="C280" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D280" s="8" t="inlineStr">
+        <is>
+          <t>Choosing the cheaper option with better features was a no-brainer.</t>
+        </is>
+      </c>
       <c r="E280" s="8" t="n"/>
       <c r="F280" s="9" t="n"/>
       <c r="G280" s="7" t="n"/>
       <c r="H280" s="8" t="n"/>
     </row>
     <row r="281">
-      <c r="A281" s="8" t="n"/>
-      <c r="B281" s="8" t="n"/>
-      <c r="C281" s="7" t="n"/>
-      <c r="D281" s="8" t="n"/>
+      <c r="A281" s="8" t="inlineStr">
+        <is>
+          <t>a shot in the dark</t>
+        </is>
+      </c>
+      <c r="B281" s="8" t="inlineStr">
+        <is>
+          <t>A wild guess or attempt with little chance of success</t>
+        </is>
+      </c>
+      <c r="C281" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D281" s="8" t="inlineStr">
+        <is>
+          <t>I don't know the answer, but I'll take a shot in the dark.</t>
+        </is>
+      </c>
       <c r="E281" s="8" t="n"/>
       <c r="F281" s="9" t="n"/>
       <c r="G281" s="7" t="n"/>
       <c r="H281" s="8" t="n"/>
     </row>
     <row r="282">
-      <c r="A282" s="8" t="n"/>
-      <c r="B282" s="8" t="n"/>
-      <c r="C282" s="7" t="n"/>
-      <c r="D282" s="8" t="n"/>
+      <c r="A282" s="8" t="inlineStr">
+        <is>
+          <t>a stone's throw away</t>
+        </is>
+      </c>
+      <c r="B282" s="8" t="inlineStr">
+        <is>
+          <t>Very close; a short distance away</t>
+        </is>
+      </c>
+      <c r="C282" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D282" s="8" t="inlineStr">
+        <is>
+          <t>The bakery is just a stone's throw away from my house.</t>
+        </is>
+      </c>
       <c r="E282" s="8" t="n"/>
       <c r="F282" s="9" t="n"/>
       <c r="G282" s="7" t="n"/>
       <c r="H282" s="8" t="n"/>
     </row>
     <row r="283">
-      <c r="A283" s="8" t="n"/>
-      <c r="B283" s="8" t="n"/>
-      <c r="C283" s="7" t="n"/>
-      <c r="D283" s="8" t="n"/>
+      <c r="A283" s="8" t="inlineStr">
+        <is>
+          <t>a wolf in sheep's clothing</t>
+        </is>
+      </c>
+      <c r="B283" s="8" t="inlineStr">
+        <is>
+          <t>A dangerous person pretending to be harmless</t>
+        </is>
+      </c>
+      <c r="C283" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D283" s="8" t="inlineStr">
+        <is>
+          <t>Be careful with him; he's a wolf in sheep's clothing.</t>
+        </is>
+      </c>
       <c r="E283" s="8" t="n"/>
       <c r="F283" s="9" t="n"/>
       <c r="G283" s="7" t="n"/>
       <c r="H283" s="8" t="n"/>
     </row>
     <row r="284">
-      <c r="A284" s="8" t="n"/>
-      <c r="B284" s="8" t="n"/>
-      <c r="C284" s="7" t="n"/>
-      <c r="D284" s="8" t="n"/>
+      <c r="A284" s="8" t="inlineStr">
+        <is>
+          <t>above board</t>
+        </is>
+      </c>
+      <c r="B284" s="8" t="inlineStr">
+        <is>
+          <t>Honest, open, and legal</t>
+        </is>
+      </c>
+      <c r="C284" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D284" s="8" t="inlineStr">
+        <is>
+          <t>All our business dealings are above board and transparent.</t>
+        </is>
+      </c>
       <c r="E284" s="8" t="n"/>
       <c r="F284" s="9" t="n"/>
       <c r="G284" s="7" t="n"/>
       <c r="H284" s="8" t="n"/>
     </row>
     <row r="285">
-      <c r="A285" s="8" t="n"/>
-      <c r="B285" s="8" t="n"/>
-      <c r="C285" s="7" t="n"/>
-      <c r="D285" s="8" t="n"/>
+      <c r="A285" s="8" t="inlineStr">
+        <is>
+          <t>actions speak louder than words</t>
+        </is>
+      </c>
+      <c r="B285" s="8" t="inlineStr">
+        <is>
+          <t>What you do is more important than what you say</t>
+        </is>
+      </c>
+      <c r="C285" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D285" s="8" t="inlineStr">
+        <is>
+          <t>He promised to help, but actions speak louder than words.</t>
+        </is>
+      </c>
       <c r="E285" s="8" t="n"/>
       <c r="F285" s="9" t="n"/>
       <c r="G285" s="7" t="n"/>
       <c r="H285" s="8" t="n"/>
     </row>
     <row r="286">
-      <c r="A286" s="8" t="n"/>
-      <c r="B286" s="8" t="n"/>
-      <c r="C286" s="7" t="n"/>
-      <c r="D286" s="8" t="n"/>
+      <c r="A286" s="8" t="inlineStr">
+        <is>
+          <t>all ears</t>
+        </is>
+      </c>
+      <c r="B286" s="8" t="inlineStr">
+        <is>
+          <t>Listening attentively and eagerly</t>
+        </is>
+      </c>
+      <c r="C286" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D286" s="8" t="inlineStr">
+        <is>
+          <t>Tell me about your trip—I'm all ears!</t>
+        </is>
+      </c>
       <c r="E286" s="8" t="n"/>
       <c r="F286" s="9" t="n"/>
       <c r="G286" s="7" t="n"/>
       <c r="H286" s="8" t="n"/>
     </row>
     <row r="287">
-      <c r="A287" s="8" t="n"/>
-      <c r="B287" s="8" t="n"/>
-      <c r="C287" s="7" t="n"/>
-      <c r="D287" s="8" t="n"/>
+      <c r="A287" s="8" t="inlineStr">
+        <is>
+          <t>apple of my eye</t>
+        </is>
+      </c>
+      <c r="B287" s="8" t="inlineStr">
+        <is>
+          <t>Someone who is cherished above all others</t>
+        </is>
+      </c>
+      <c r="C287" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D287" s="8" t="inlineStr">
+        <is>
+          <t>His youngest daughter is the apple of his eye.</t>
+        </is>
+      </c>
       <c r="E287" s="8" t="n"/>
       <c r="F287" s="9" t="n"/>
       <c r="G287" s="7" t="n"/>
       <c r="H287" s="8" t="n"/>
     </row>
     <row r="288">
-      <c r="A288" s="8" t="n"/>
-      <c r="B288" s="8" t="n"/>
-      <c r="C288" s="7" t="n"/>
-      <c r="D288" s="8" t="n"/>
+      <c r="A288" s="8" t="inlineStr">
+        <is>
+          <t>at the drop of a hat</t>
+        </is>
+      </c>
+      <c r="B288" s="8" t="inlineStr">
+        <is>
+          <t>Immediately, without hesitation</t>
+        </is>
+      </c>
+      <c r="C288" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D288" s="8" t="inlineStr">
+        <is>
+          <t>She would travel to Paris at the drop of a hat if she had the money.</t>
+        </is>
+      </c>
       <c r="E288" s="8" t="n"/>
       <c r="F288" s="9" t="n"/>
       <c r="G288" s="7" t="n"/>
       <c r="H288" s="8" t="n"/>
     </row>
     <row r="289">
-      <c r="A289" s="8" t="n"/>
-      <c r="B289" s="8" t="n"/>
-      <c r="C289" s="7" t="n"/>
-      <c r="D289" s="8" t="n"/>
+      <c r="A289" s="8" t="inlineStr">
+        <is>
+          <t>at the eleventh hour</t>
+        </is>
+      </c>
+      <c r="B289" s="8" t="inlineStr">
+        <is>
+          <t>At the last possible moment</t>
+        </is>
+      </c>
+      <c r="C289" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D289" s="8" t="inlineStr">
+        <is>
+          <t>He finished his project at the eleventh hour.</t>
+        </is>
+      </c>
       <c r="E289" s="8" t="n"/>
       <c r="F289" s="9" t="n"/>
       <c r="G289" s="7" t="n"/>
       <c r="H289" s="8" t="n"/>
     </row>
     <row r="290">
-      <c r="A290" s="8" t="n"/>
-      <c r="B290" s="8" t="n"/>
-      <c r="C290" s="7" t="n"/>
-      <c r="D290" s="8" t="n"/>
+      <c r="A290" s="8" t="inlineStr">
+        <is>
+          <t>back to square one</t>
+        </is>
+      </c>
+      <c r="B290" s="8" t="inlineStr">
+        <is>
+          <t>Back to the beginning after a failed attempt</t>
+        </is>
+      </c>
+      <c r="C290" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D290" s="8" t="inlineStr">
+        <is>
+          <t>The plan didn't work, so we're back to square one.</t>
+        </is>
+      </c>
       <c r="E290" s="8" t="n"/>
       <c r="F290" s="9" t="n"/>
       <c r="G290" s="7" t="n"/>
       <c r="H290" s="8" t="n"/>
     </row>
     <row r="291">
-      <c r="A291" s="8" t="n"/>
-      <c r="B291" s="8" t="n"/>
-      <c r="C291" s="7" t="n"/>
-      <c r="D291" s="8" t="n"/>
+      <c r="A291" s="8" t="inlineStr">
+        <is>
+          <t>bend over backwards</t>
+        </is>
+      </c>
+      <c r="B291" s="8" t="inlineStr">
+        <is>
+          <t>To try very hard to help or please someone</t>
+        </is>
+      </c>
+      <c r="C291" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D291" s="8" t="inlineStr">
+        <is>
+          <t>My parents bent over backwards to support my education.</t>
+        </is>
+      </c>
       <c r="E291" s="8" t="n"/>
       <c r="F291" s="9" t="n"/>
       <c r="G291" s="7" t="n"/>
       <c r="H291" s="8" t="n"/>
     </row>
     <row r="292">
-      <c r="A292" s="8" t="n"/>
-      <c r="B292" s="8" t="n"/>
-      <c r="C292" s="7" t="n"/>
-      <c r="D292" s="8" t="n"/>
+      <c r="A292" s="8" t="inlineStr">
+        <is>
+          <t>better late than never</t>
+        </is>
+      </c>
+      <c r="B292" s="8" t="inlineStr">
+        <is>
+          <t>It's better to do something late than not at all</t>
+        </is>
+      </c>
+      <c r="C292" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D292" s="8" t="inlineStr">
+        <is>
+          <t>He finally apologized—better late than never.</t>
+        </is>
+      </c>
       <c r="E292" s="8" t="n"/>
       <c r="F292" s="9" t="n"/>
       <c r="G292" s="7" t="n"/>
       <c r="H292" s="8" t="n"/>
     </row>
     <row r="293">
-      <c r="A293" s="8" t="n"/>
-      <c r="B293" s="8" t="n"/>
-      <c r="C293" s="7" t="n"/>
-      <c r="D293" s="8" t="n"/>
+      <c r="A293" s="8" t="inlineStr">
+        <is>
+          <t>better safe than sorry</t>
+        </is>
+      </c>
+      <c r="B293" s="8" t="inlineStr">
+        <is>
+          <t>It's wise to be cautious rather than regret something later</t>
+        </is>
+      </c>
+      <c r="C293" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D293" s="8" t="inlineStr">
+        <is>
+          <t>I always lock my car; better safe than sorry.</t>
+        </is>
+      </c>
       <c r="E293" s="8" t="n"/>
       <c r="F293" s="9" t="n"/>
       <c r="G293" s="7" t="n"/>
       <c r="H293" s="8" t="n"/>
     </row>
     <row r="294">
-      <c r="A294" s="8" t="n"/>
-      <c r="B294" s="8" t="n"/>
-      <c r="C294" s="7" t="n"/>
-      <c r="D294" s="8" t="n"/>
+      <c r="A294" s="8" t="inlineStr">
+        <is>
+          <t>bite the dust</t>
+        </is>
+      </c>
+      <c r="B294" s="8" t="inlineStr">
+        <is>
+          <t>To fail, die, or be defeated</t>
+        </is>
+      </c>
+      <c r="C294" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D294" s="8" t="inlineStr">
+        <is>
+          <t>Another one of my plants bit the dust this week.</t>
+        </is>
+      </c>
       <c r="E294" s="8" t="n"/>
       <c r="F294" s="9" t="n"/>
       <c r="G294" s="7" t="n"/>
       <c r="H294" s="8" t="n"/>
     </row>
     <row r="295">
-      <c r="A295" s="8" t="n"/>
-      <c r="B295" s="8" t="n"/>
-      <c r="C295" s="7" t="n"/>
-      <c r="D295" s="8" t="n"/>
+      <c r="A295" s="8" t="inlineStr">
+        <is>
+          <t>blow your mind</t>
+        </is>
+      </c>
+      <c r="B295" s="8" t="inlineStr">
+        <is>
+          <t>To amaze or astonish you</t>
+        </is>
+      </c>
+      <c r="C295" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D295" s="8" t="inlineStr">
+        <is>
+          <t>The magician's tricks will blow your mind.</t>
+        </is>
+      </c>
       <c r="E295" s="8" t="n"/>
       <c r="F295" s="9" t="n"/>
       <c r="G295" s="7" t="n"/>
       <c r="H295" s="8" t="n"/>
     </row>
     <row r="296">
-      <c r="A296" s="8" t="n"/>
-      <c r="B296" s="8" t="n"/>
-      <c r="C296" s="7" t="n"/>
-      <c r="D296" s="8" t="n"/>
+      <c r="A296" s="8" t="inlineStr">
+        <is>
+          <t>break a leg</t>
+        </is>
+      </c>
+      <c r="B296" s="8" t="inlineStr">
+        <is>
+          <t>Good luck (especially before a performance)</t>
+        </is>
+      </c>
+      <c r="C296" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D296" s="8" t="inlineStr">
+        <is>
+          <t>Break a leg at your audition tonight!</t>
+        </is>
+      </c>
       <c r="E296" s="8" t="n"/>
       <c r="F296" s="9" t="n"/>
       <c r="G296" s="7" t="n"/>
       <c r="H296" s="8" t="n"/>
     </row>
     <row r="297">
-      <c r="A297" s="8" t="n"/>
-      <c r="B297" s="8" t="n"/>
-      <c r="C297" s="7" t="n"/>
-      <c r="D297" s="8" t="n"/>
+      <c r="A297" s="8" t="inlineStr">
+        <is>
+          <t>bring home the bacon</t>
+        </is>
+      </c>
+      <c r="B297" s="8" t="inlineStr">
+        <is>
+          <t>To earn money to support the family</t>
+        </is>
+      </c>
+      <c r="C297" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D297" s="8" t="inlineStr">
+        <is>
+          <t>She works two jobs to bring home the bacon.</t>
+        </is>
+      </c>
       <c r="E297" s="8" t="n"/>
       <c r="F297" s="9" t="n"/>
       <c r="G297" s="7" t="n"/>
       <c r="H297" s="8" t="n"/>
     </row>
     <row r="298">
-      <c r="A298" s="8" t="n"/>
-      <c r="B298" s="8" t="n"/>
-      <c r="C298" s="7" t="n"/>
-      <c r="D298" s="8" t="n"/>
+      <c r="A298" s="8" t="inlineStr">
+        <is>
+          <t>burn the candle at both ends</t>
+        </is>
+      </c>
+      <c r="B298" s="8" t="inlineStr">
+        <is>
+          <t>To work too hard by doing too many things</t>
+        </is>
+      </c>
+      <c r="C298" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D298" s="8" t="inlineStr">
+        <is>
+          <t>If you keep burning the candle at both ends, you'll get sick.</t>
+        </is>
+      </c>
       <c r="E298" s="8" t="n"/>
       <c r="F298" s="9" t="n"/>
       <c r="G298" s="7" t="n"/>
       <c r="H298" s="8" t="n"/>
     </row>
     <row r="299">
-      <c r="A299" s="8" t="n"/>
-      <c r="B299" s="8" t="n"/>
-      <c r="C299" s="7" t="n"/>
-      <c r="D299" s="8" t="n"/>
+      <c r="A299" s="8" t="inlineStr">
+        <is>
+          <t>bury the hatchet</t>
+        </is>
+      </c>
+      <c r="B299" s="8" t="inlineStr">
+        <is>
+          <t>To make peace after an argument or dispute</t>
+        </is>
+      </c>
+      <c r="C299" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D299" s="8" t="inlineStr">
+        <is>
+          <t>After years of fighting, the brothers finally buried the hatchet.</t>
+        </is>
+      </c>
       <c r="E299" s="8" t="n"/>
       <c r="F299" s="9" t="n"/>
       <c r="G299" s="7" t="n"/>
       <c r="H299" s="8" t="n"/>
     </row>
     <row r="300">
-      <c r="A300" s="8" t="n"/>
-      <c r="B300" s="8" t="n"/>
-      <c r="C300" s="7" t="n"/>
-      <c r="D300" s="8" t="n"/>
+      <c r="A300" s="8" t="inlineStr">
+        <is>
+          <t>by the skin of your teeth</t>
+        </is>
+      </c>
+      <c r="B300" s="8" t="inlineStr">
+        <is>
+          <t>Just barely; narrowly</t>
+        </is>
+      </c>
+      <c r="C300" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D300" s="8" t="inlineStr">
+        <is>
+          <t>I passed the exam by the skin of my teeth.</t>
+        </is>
+      </c>
       <c r="E300" s="8" t="n"/>
       <c r="F300" s="9" t="n"/>
       <c r="G300" s="7" t="n"/>
       <c r="H300" s="8" t="n"/>
     </row>
     <row r="301">
-      <c r="A301" s="8" t="n"/>
-      <c r="B301" s="8" t="n"/>
-      <c r="C301" s="7" t="n"/>
-      <c r="D301" s="8" t="n"/>
+      <c r="A301" s="8" t="inlineStr">
+        <is>
+          <t>call it a day</t>
+        </is>
+      </c>
+      <c r="B301" s="8" t="inlineStr">
+        <is>
+          <t>To stop working for the day</t>
+        </is>
+      </c>
+      <c r="C301" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D301" s="8" t="inlineStr">
+        <is>
+          <t>It's getting late; let's call it a day.</t>
+        </is>
+      </c>
       <c r="E301" s="8" t="n"/>
       <c r="F301" s="9" t="n"/>
       <c r="G301" s="7" t="n"/>
       <c r="H301" s="8" t="n"/>
     </row>
     <row r="302">
-      <c r="A302" s="8" t="n"/>
-      <c r="B302" s="8" t="n"/>
-      <c r="C302" s="7" t="n"/>
-      <c r="D302" s="8" t="n"/>
+      <c r="A302" s="8" t="inlineStr">
+        <is>
+          <t>can of worms</t>
+        </is>
+      </c>
+      <c r="B302" s="8" t="inlineStr">
+        <is>
+          <t>A complicated situation that creates more problems</t>
+        </is>
+      </c>
+      <c r="C302" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D302" s="8" t="inlineStr">
+        <is>
+          <t>Mentioning his ex opened a whole can of worms.</t>
+        </is>
+      </c>
       <c r="E302" s="8" t="n"/>
       <c r="F302" s="9" t="n"/>
       <c r="G302" s="7" t="n"/>
       <c r="H302" s="8" t="n"/>
     </row>
     <row r="303">
-      <c r="A303" s="8" t="n"/>
-      <c r="B303" s="8" t="n"/>
-      <c r="C303" s="7" t="n"/>
-      <c r="D303" s="8" t="n"/>
+      <c r="A303" s="8" t="inlineStr">
+        <is>
+          <t>catch-22</t>
+        </is>
+      </c>
+      <c r="B303" s="8" t="inlineStr">
+        <is>
+          <t>A no-win situation with contradictory rules</t>
+        </is>
+      </c>
+      <c r="C303" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D303" s="8" t="inlineStr">
+        <is>
+          <t>You need experience to get a job, but you need a job to get experience—it's a catch-22.</t>
+        </is>
+      </c>
       <c r="E303" s="8" t="n"/>
       <c r="F303" s="9" t="n"/>
       <c r="G303" s="7" t="n"/>
       <c r="H303" s="8" t="n"/>
     </row>
     <row r="304">
-      <c r="A304" s="8" t="n"/>
-      <c r="B304" s="8" t="n"/>
-      <c r="C304" s="7" t="n"/>
-      <c r="D304" s="8" t="n"/>
+      <c r="A304" s="8" t="inlineStr">
+        <is>
+          <t>caught red-handed</t>
+        </is>
+      </c>
+      <c r="B304" s="8" t="inlineStr">
+        <is>
+          <t>Caught in the act of doing something wrong</t>
+        </is>
+      </c>
+      <c r="C304" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D304" s="8" t="inlineStr">
+        <is>
+          <t>The thief was caught red-handed stealing from the store.</t>
+        </is>
+      </c>
       <c r="E304" s="8" t="n"/>
       <c r="F304" s="9" t="n"/>
       <c r="G304" s="7" t="n"/>
       <c r="H304" s="8" t="n"/>
     </row>
     <row r="305">
-      <c r="A305" s="8" t="n"/>
-      <c r="B305" s="8" t="n"/>
-      <c r="C305" s="7" t="n"/>
-      <c r="D305" s="8" t="n"/>
+      <c r="A305" s="8" t="inlineStr">
+        <is>
+          <t>chew the fat</t>
+        </is>
+      </c>
+      <c r="B305" s="8" t="inlineStr">
+        <is>
+          <t>To chat casually for a long time</t>
+        </is>
+      </c>
+      <c r="C305" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D305" s="8" t="inlineStr">
+        <is>
+          <t>We sat on the porch and chewed the fat for hours.</t>
+        </is>
+      </c>
       <c r="E305" s="8" t="n"/>
       <c r="F305" s="9" t="n"/>
       <c r="G305" s="7" t="n"/>
       <c r="H305" s="8" t="n"/>
     </row>
     <row r="306">
-      <c r="A306" s="8" t="n"/>
-      <c r="B306" s="8" t="n"/>
-      <c r="C306" s="7" t="n"/>
-      <c r="D306" s="8" t="n"/>
+      <c r="A306" s="8" t="inlineStr">
+        <is>
+          <t>clear the air</t>
+        </is>
+      </c>
+      <c r="B306" s="8" t="inlineStr">
+        <is>
+          <t>To resolve a misunderstanding or conflict</t>
+        </is>
+      </c>
+      <c r="C306" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D306" s="8" t="inlineStr">
+        <is>
+          <t>Let's clear the air and talk about what happened.</t>
+        </is>
+      </c>
       <c r="E306" s="8" t="n"/>
       <c r="F306" s="9" t="n"/>
       <c r="G306" s="7" t="n"/>
       <c r="H306" s="8" t="n"/>
     </row>
     <row r="307">
-      <c r="A307" s="8" t="n"/>
-      <c r="B307" s="8" t="n"/>
-      <c r="C307" s="7" t="n"/>
-      <c r="D307" s="8" t="n"/>
+      <c r="A307" s="8" t="inlineStr">
+        <is>
+          <t>close call</t>
+        </is>
+      </c>
+      <c r="B307" s="8" t="inlineStr">
+        <is>
+          <t>A narrow escape from danger or trouble</t>
+        </is>
+      </c>
+      <c r="C307" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D307" s="8" t="inlineStr">
+        <is>
+          <t>That was a close call! The car almost hit us.</t>
+        </is>
+      </c>
       <c r="E307" s="8" t="n"/>
       <c r="F307" s="9" t="n"/>
       <c r="G307" s="7" t="n"/>
       <c r="H307" s="8" t="n"/>
     </row>
     <row r="308">
-      <c r="A308" s="8" t="n"/>
-      <c r="B308" s="8" t="n"/>
-      <c r="C308" s="7" t="n"/>
-      <c r="D308" s="8" t="n"/>
+      <c r="A308" s="8" t="inlineStr">
+        <is>
+          <t>cold turkey</t>
+        </is>
+      </c>
+      <c r="B308" s="8" t="inlineStr">
+        <is>
+          <t>To stop an addiction abruptly, without help</t>
+        </is>
+      </c>
+      <c r="C308" s="7" t="inlineStr">
+        <is>
+          <t>idiom</t>
+        </is>
+      </c>
+      <c r="D308" s="8" t="inlineStr">
+        <is>
+          <t>He quit smoking cold turkey last year.</t>
+        </is>
+      </c>
       <c r="E308" s="8" t="n"/>
       <c r="F308" s="9" t="n"/>
       <c r="G308" s="7" t="n"/>

</xml_diff>